<commit_message>
update template indikator 1 & 6
</commit_message>
<xml_diff>
--- a/public/templates/Indikator 1_Kejuaraan Pelajar Tingkat Nasional dan Internasional.xlsx
+++ b/public/templates/Indikator 1_Kejuaraan Pelajar Tingkat Nasional dan Internasional.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kuliah\Semester 6\PKL\arindama\Spreadsheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{403B10DB-27C4-4532-A648-869E6CA1ACE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C528B5-6E0B-4625-8AFB-0BC2AEAA04D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F0869B6-331C-4543-BA84-824070015A42}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>Nama Kegiatan/ Kejuaraan Olahraga</t>
   </si>
@@ -92,6 +92,9 @@
   </si>
   <si>
     <t>Mandiri</t>
+  </si>
+  <si>
+    <t>Partisipan</t>
   </si>
 </sst>
 </file>
@@ -1299,9 +1302,9 @@
           </x14:formula1>
           <xm:sqref>D2:D100</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pilih medali yang didapatkan" prompt="Pilih medali berdasarkan dropdown menu" xr:uid="{3F8BBAEF-7044-4FED-AE1C-E24D96068BC4}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Pilih medali yang didapatkan" prompt="Pilih medali berdasarkan opsi dropdown menu" xr:uid="{3F8BBAEF-7044-4FED-AE1C-E24D96068BC4}">
           <x14:formula1>
-            <xm:f>Sheet2!$E$2:$E$4</xm:f>
+            <xm:f>Sheet2!$E$2:$E$5</xm:f>
           </x14:formula1>
           <xm:sqref>E2:E100</xm:sqref>
         </x14:dataValidation>
@@ -1369,6 +1372,9 @@
       <c r="C5" t="s">
         <v>13</v>
       </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="C6" t="s">

</xml_diff>